<commit_message>
Rewrite Core 2 for Copilot Chat and first-time users
Drexel does not have the Microsoft 365 Copilot license, so Core 2 now
uses only Copilot Chat and ChatGPT Edu (paste or upload, then copy the
answer back). Simplified to follow directly from Core 1: guided upload,
three everyday jobs, own task saved as a recipe. Page, HTML slides,
PowerPoint (20 slides, with build script), instructor guide, and demo
file wording updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-materials/Workshop2_Demo_SeminarAttendance.xlsx
+++ b/demo-materials/Workshop2_Demo_SeminarAttendance.xlsx
@@ -77,7 +77,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Demo file for AI Workshops for DSPH - Workshop 2, Track C (Excel).</t>
+    <t xml:space="preserve">Demo file for AI Workshops for DSPH - Workshop 2, Track C (Make sense of a spreadsheet).</t>
   </si>
   <si>
     <t xml:space="preserve">Synthetic data: monthly seminar attendance and catering cost for three departments, AY 2025-26.</t>
@@ -86,19 +86,19 @@
     <t xml:space="preserve">All values are fictional and non-sensitive.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prompts to try with Copilot in Excel:</t>
+    <t xml:space="preserve">Prompts to try (upload this file to Copilot Chat or ChatGPT Edu):</t>
   </si>
   <si>
     <t xml:space="preserve">1. Summarize this data. What stands out?</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Add a column that flags rows where cost per attendee is over $12.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Suggest a chart showing the attendance trend by department across the year.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify step: check the flag formula against one row by hand before trusting the column.</t>
+    <t xml:space="preserve">2. Write an Excel formula for a new column E that says "Over" when cost per attendee is more than $12. Tell me how to copy it down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Which months had the lowest attendance? Suggest one chart I could make in Excel to show the trend.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify step: paste the formula into Excel, check one row by hand, and count the flagged rows.</t>
   </si>
 </sst>
 </file>

</xml_diff>